<commit_message>
📅 日报更新 2026-08-20 07:04
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-08-20.xlsx
+++ b/data/exports/黄老师/dist_order_2026-08-20.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>49415939</v>
+        <v>49432023</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>花生米</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-20 11:55:45</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,17 +164,17 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>49415918</v>
+        <v>49415939</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>杨梅芳</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-19 22:48:58</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>49415913</v>
+        <v>49415918</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>心语无言</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-19 22:48:24</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>49415890</v>
+        <v>49415913</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>安好</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-19 22:48:18</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -360,21 +360,16 @@
       <c r="L5" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N5" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>49415874</v>
+        <v>49415890</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>雨夜聆风</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -399,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-19 22:47:56</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,16 +420,21 @@
       <c r="L6" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N6" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>49415871</v>
+        <v>49415874</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>飘</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -459,7 +459,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-19 22:47:40</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -490,59 +490,119 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L8" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="0">
         <v>49415867</v>
       </c>
-      <c r="B8" s="0" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D8" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E8" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F8" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G8" s="0" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="0" t="inlineStr">
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
         <is>
           <t>黄老师-抖音01</t>
         </is>
       </c>
-      <c r="J8" s="0" t="inlineStr">
+      <c r="J9" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K8" s="0" t="inlineStr">
+      <c r="K9" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L8" s="0" t="inlineStr">
+      <c r="L9" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>